<commit_message>
Update sample Excel files with po_number and date_of_reporting columns
- Add date_of_reporting alias to Excel parser for upload support
- Add po_number and date_of_reporting columns to sample rate card generator
- Regenerate TestRateCard.xlsx with all 9 columns

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/TestRateCard.xlsx
+++ b/data/TestRateCard.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Rate Card" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="29">
   <si>
     <t>client_name</t>
   </si>
@@ -34,6 +34,12 @@
     <t>leaves_allowed</t>
   </si>
   <si>
+    <t>po_number</t>
+  </si>
+  <si>
+    <t>date_of_reporting</t>
+  </si>
+  <si>
     <t>Acme Corp</t>
   </si>
   <si>
@@ -49,6 +55,9 @@
     <t>Bob Smith</t>
   </si>
   <si>
+    <t>PO-2025-001</t>
+  </si>
+  <si>
     <t>EMP002</t>
   </si>
   <si>
@@ -67,6 +76,9 @@
     <t>2024-06-01</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>EMP004</t>
   </si>
   <si>
@@ -74,6 +86,9 @@
   </si>
   <si>
     <t>2022-11-10</t>
+  </si>
+  <si>
+    <t>PO-2025-002</t>
   </si>
   <si>
     <t>EMP005</t>
@@ -89,7 +104,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -97,13 +112,22 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2F5496"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -118,8 +142,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -459,47 +486,63 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="9" width="18" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F2">
         <v>50000</v>
@@ -507,22 +550,28 @@
       <c r="G2">
         <v>2</v>
       </c>
+      <c r="H2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s">
         <v>13</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
       </c>
       <c r="F3">
         <v>60000</v>
@@ -530,22 +579,28 @@
       <c r="G3">
         <v>1</v>
       </c>
+      <c r="H3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I3" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F4">
         <v>45000</v>
@@ -553,22 +608,28 @@
       <c r="G4">
         <v>2</v>
       </c>
+      <c r="H4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F5">
         <v>70000</v>
@@ -576,22 +637,28 @@
       <c r="G5">
         <v>3</v>
       </c>
+      <c r="H5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I5" t="s">
+        <v>24</v>
+      </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="D6" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="E6" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F6">
         <v>55000</v>
@@ -599,8 +666,15 @@
       <c r="G6">
         <v>2</v>
       </c>
+      <c r="H6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I6" t="s">
+        <v>28</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>